<commit_message>
Unicorn city ranking on founded-OR-HQ basis (label + dedup)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UK-tech-data.xlsx
+++ b/UK-tech-data.xlsx
@@ -5673,7 +5673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5691,7 +5691,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Verified unicorns &amp; $1B exits headquartered in each UK city.</t>
+          <t>Verified unicorns &amp; $1B exits, founded-or-HQ basis, by UK city. (UK-founded unicorns now HQ'd abroad have no UK city and sit in the national total.)</t>
         </is>
       </c>
     </row>
@@ -5744,7 +5744,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Manchester</t>
+          <t>Oxford</t>
         </is>
       </c>
       <c r="C7" s="12" t="n">
@@ -5757,7 +5757,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Oxford</t>
+          <t>Manchester</t>
         </is>
       </c>
       <c r="C8" s="12" t="n">
@@ -5770,7 +5770,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Reigate</t>
+          <t>Milton</t>
         </is>
       </c>
       <c r="C9" s="12" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bristol</t>
+          <t>Reigate</t>
         </is>
       </c>
       <c r="C10" s="12" t="n">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Sheffield</t>
+          <t>Leeds</t>
         </is>
       </c>
       <c r="C11" s="12" t="n">
@@ -5809,7 +5809,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Milton</t>
+          <t>Nottingham</t>
         </is>
       </c>
       <c r="C12" s="12" t="n">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Leeds</t>
+          <t>Sheffield</t>
         </is>
       </c>
       <c r="C13" s="12" t="n">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nottingham</t>
+          <t>Bristol</t>
         </is>
       </c>
       <c r="C14" s="12" t="n">
@@ -5848,7 +5848,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hatfield</t>
+          <t>Babraham</t>
         </is>
       </c>
       <c r="C15" s="12" t="n">
@@ -5861,7 +5861,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Babraham</t>
+          <t>Horsham</t>
         </is>
       </c>
       <c r="C16" s="12" t="n">
@@ -5874,36 +5874,10 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Horsham</t>
+          <t>Crewe</t>
         </is>
       </c>
       <c r="C17" s="12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Crewe</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Cheltenham</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Briefing for Rowland Manthorpe: factual copy, metro unicorns, share as bar, bar totals
- Remove political/editorial commentary; keep commentary factual
- UK regional unicorns by metro area (founded-OR-HQ); London = London metro
- UK share of European VC as bar chart, y-axis from zero
- Totals on all annual bars and unicorn bars
- Source lines reduced to 'Source: Dealroom.co'

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UK-tech-data.xlsx
+++ b/UK-tech-data.xlsx
@@ -14,7 +14,7 @@
     <sheet name="AI VC quarterly" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Shares" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Unicorns by country" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="UK unicorn cities" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="UK unicorn metros" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="UK cities by VC" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="UK cities by AI VC" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
@@ -657,7 +657,7 @@
     <row r="23">
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>•  Even excluding London, the rest of the UK (76 unicorns) would out-rank France, Sweden and Australia.</t>
+          <t>•  Excluding the London metro, the rest of the UK (64 unicorns) ranks ahead of Sweden and Australia.</t>
         </is>
       </c>
     </row>
@@ -5611,29 +5611,29 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="n">
+      <c r="A12" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>United Kingdom (ex-London)</t>
         </is>
       </c>
-      <c r="C12" s="14" t="n">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="n">
-        <v>66</v>
+      <c r="C13" s="14" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="14">
@@ -5673,7 +5673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5684,14 +5684,14 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>UK cities by number of unicorns</t>
+          <t>UK metro areas by number of unicorns</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Verified unicorns &amp; $1B exits, founded-or-HQ basis, by UK city. (UK-founded unicorns now HQ'd abroad have no UK city and sit in the national total.)</t>
+          <t>Verified unicorns &amp; $1B exits, founded-or-HQ basis, by UK metro area (satellite towns rolled into their metro).</t>
         </is>
       </c>
     </row>
@@ -5703,7 +5703,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>City</t>
+          <t>Metro</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -5722,7 +5722,7 @@
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>143</v>
+        <v>155</v>
       </c>
     </row>
     <row r="6">
@@ -5735,7 +5735,7 @@
         </is>
       </c>
       <c r="C6" s="12" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -5744,11 +5744,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Oxford</t>
+          <t>Manchester</t>
         </is>
       </c>
       <c r="C7" s="12" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -5757,11 +5757,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Manchester</t>
+          <t>Oxford</t>
         </is>
       </c>
       <c r="C8" s="12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -5770,7 +5770,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Milton</t>
+          <t>Nottingham</t>
         </is>
       </c>
       <c r="C9" s="12" t="n">
@@ -5783,7 +5783,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Reigate</t>
+          <t>Birmingham</t>
         </is>
       </c>
       <c r="C10" s="12" t="n">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Leeds</t>
+          <t>Bristol</t>
         </is>
       </c>
       <c r="C11" s="12" t="n">
@@ -5809,7 +5809,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Nottingham</t>
+          <t>Sheffield</t>
         </is>
       </c>
       <c r="C12" s="12" t="n">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sheffield</t>
+          <t>Leeds–Bradford</t>
         </is>
       </c>
       <c r="C13" s="12" t="n">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bristol</t>
+          <t>Edinburgh</t>
         </is>
       </c>
       <c r="C14" s="12" t="n">
@@ -5848,7 +5848,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Babraham</t>
+          <t>Windsor-Maidenhead</t>
         </is>
       </c>
       <c r="C15" s="12" t="n">
@@ -5861,7 +5861,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Horsham</t>
+          <t>Newcastle upon Tyne</t>
         </is>
       </c>
       <c r="C16" s="12" t="n">
@@ -5874,10 +5874,23 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Crewe</t>
+          <t>Glasgow</t>
         </is>
       </c>
       <c r="C17" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Cardiff-Newport</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Metro treatment for VC, drop stat boxes, dated as-of, split AI charts
- UK VC + AI VC by metro area (fan-out over metro location ids)
- Remove hero KPI stat boxes
- '2026 data is to 25 June 2026' (explicit date, not 'year-to-date')
- Split AI into two charts: AI VC funding ($B) and AI share of UK VC (%)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UK-tech-data.xlsx
+++ b/UK-tech-data.xlsx
@@ -15,8 +15,8 @@
     <sheet name="Shares" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Unicorns by country" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="UK unicorn metros" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="UK cities by VC" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="UK cities by AI VC" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="UK metros by VC" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="UK metros by AI VC" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -694,21 +694,21 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>UK cities by AI VC funding (annual)</t>
+          <t>UK metro areas by AI VC funding (annual)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Top cities by AI VC raised, $B per year.</t>
+          <t>Top metro areas by AI VC raised, $B per year.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>City</t>
+          <t>Metro</t>
         </is>
       </c>
       <c r="B4" s="7" t="n">
@@ -842,7 +842,7 @@
         <v>0</v>
       </c>
       <c r="N6" s="10" t="n">
-        <v>2.89</v>
+        <v>3.16</v>
       </c>
     </row>
     <row r="7">
@@ -888,7 +888,7 @@
         <v>0</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>2.32</v>
+        <v>2.51</v>
       </c>
     </row>
     <row r="8">
@@ -980,7 +980,7 @@
         <v>0</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>0.63</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="10">
@@ -1032,7 +1032,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Altrincham</t>
+          <t>Birmingham</t>
         </is>
       </c>
       <c r="B11" s="8" t="n">
@@ -1072,13 +1072,13 @@
         <v>0</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>0.33</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Birmingham</t>
+          <t>Glasgow</t>
         </is>
       </c>
       <c r="B12" s="8" t="n">
@@ -1118,13 +1118,13 @@
         <v>0</v>
       </c>
       <c r="N12" s="10" t="n">
-        <v>0.33</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Wallingford</t>
+          <t>Leeds–Bradford</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
@@ -1164,13 +1164,13 @@
         <v>0</v>
       </c>
       <c r="N13" s="10" t="n">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Milton</t>
+          <t>Belfast</t>
         </is>
       </c>
       <c r="B14" s="8" t="n">
@@ -1210,13 +1210,13 @@
         <v>0</v>
       </c>
       <c r="N14" s="10" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Glasgow</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B15" s="8" t="n">
@@ -1256,13 +1256,13 @@
         <v>0</v>
       </c>
       <c r="N15" s="10" t="n">
-        <v>0.16</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Milton Keynes</t>
+          <t>Cardiff-Newport</t>
         </is>
       </c>
       <c r="B16" s="8" t="n">
@@ -1302,7 +1302,7 @@
         <v>0</v>
       </c>
       <c r="N16" s="10" t="n">
-        <v>0.15</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -5927,21 +5927,21 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>UK cities by VC funding (annual)</t>
+          <t>UK metro areas by VC funding (annual)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Top cities by total VC raised, $B per year.</t>
+          <t>Top metro areas by total VC raised, $B per year.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>City</t>
+          <t>Metro</t>
         </is>
       </c>
       <c r="B4" s="7" t="n">
@@ -6075,7 +6075,7 @@
         <v>0</v>
       </c>
       <c r="N6" s="10" t="n">
-        <v>10.19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -6121,7 +6121,7 @@
         <v>0</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>5.45</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -6167,7 +6167,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="10" t="n">
-        <v>3.12</v>
+        <v>4.25</v>
       </c>
     </row>
     <row r="9">
@@ -6213,7 +6213,7 @@
         <v>0</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>2.91</v>
+        <v>2.94</v>
       </c>
     </row>
     <row r="10">
@@ -6259,13 +6259,13 @@
         <v>0</v>
       </c>
       <c r="N10" s="10" t="n">
-        <v>2.16</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Milton</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B11" s="8" t="n">
@@ -6305,13 +6305,13 @@
         <v>0</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>1.53</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Reading</t>
+          <t>Glasgow</t>
         </is>
       </c>
       <c r="B12" s="8" t="n">
@@ -6351,13 +6351,13 @@
         <v>0</v>
       </c>
       <c r="N12" s="10" t="n">
-        <v>1.37</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Loughborough</t>
+          <t>Leeds–Bradford</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
@@ -6397,13 +6397,13 @@
         <v>0</v>
       </c>
       <c r="N13" s="10" t="n">
-        <v>1.32</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Stevenage</t>
+          <t>Birmingham</t>
         </is>
       </c>
       <c r="B14" s="8" t="n">
@@ -6443,13 +6443,13 @@
         <v>0</v>
       </c>
       <c r="N14" s="10" t="n">
-        <v>1.22</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Leeds</t>
+          <t>Newcastle upon Tyne</t>
         </is>
       </c>
       <c r="B15" s="8" t="n">
@@ -6489,13 +6489,13 @@
         <v>0</v>
       </c>
       <c r="N15" s="10" t="n">
-        <v>1.03</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Billingham</t>
+          <t>Cardiff-Newport</t>
         </is>
       </c>
       <c r="B16" s="8" t="n">
@@ -6535,7 +6535,7 @@
         <v>0</v>
       </c>
       <c r="N16" s="10" t="n">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add top 10 UK VC rounds for 2025 and 2026
New section + workbook 'Top rounds' tab. is_vc_round filter excludes debt/M&A/IPO; lead investors first.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UK-tech-data.xlsx
+++ b/UK-tech-data.xlsx
@@ -17,6 +17,7 @@
     <sheet name="UK unicorn metros" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="UK metros by VC" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="UK metros by AI VC" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Top rounds" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +29,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,6 +58,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000B1F3A"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="5">
@@ -94,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -116,6 +122,7 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1310,6 +1317,676 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Largest UK VC rounds</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Top 10 VC rounds by deal size, 2025 and 2026 year-to-date (to 25 June 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Amount ($m)</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Lead investors</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Revolut</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Late VC</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Mubadala Capital</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Nscale</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Series B</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Aker ASA, G Squared, Nvidia</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Kraken</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Early VC</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>12/2025</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>D1 Capital Partners, Ontario Teachers’ Pension Plan, Durable Capital Partners</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>CityFibre</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>660</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Growth Equity VC</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>07/2025</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Antin Infrastructure Partners, Mubadala Capital, Interogo Holding</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>FNZ</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>650</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Growth Equity VC</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>11/2025</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Ninety One, Nucleus Financial, Aberdeen</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Quantinuum</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>600</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Late VC</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>09/2025</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Quanta Computer, NVentures, QED Investors</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Isomorphic Labs</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>600</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Late VC</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Thrive Capital, GV</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Rapyd</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>500</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Series F</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>XBO.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>FNZ</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>500</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Growth Equity VC</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Nscale</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>433</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Late VC</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Nvidia, Dell Technologies Capital, Blue Owl Capital</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Amount ($m)</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Lead investors</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Isomorphic Labs</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="n">
+        <v>2100</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Series B</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Thrive Capital, UK Sovereign AI, GV</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Nscale</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Series C</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Aker ASA, 8090 Industries, Dell</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Wayve</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Series D</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>SoftBank Vision Fund, Eclipse Ventures, Balderton Capital</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Ineffable Intelligence</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Sequoia, Lightspeed Venture Partners, Government of the United Kingdom</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Recursive Superintelligence</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="n">
+        <v>650</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>GV, Nvidia, Greycroft Partners</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>6</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="n">
+        <v>500</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Series D</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>02/2026</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Sequoia, Smash Capital, ICONIQ Capital</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>7</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>CuspAI</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Late VC</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>06/2026</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Kleiner Perkins, Bezos Expeditions</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>8</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Oxford Quantum Circuits</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="n">
+        <v>350</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Series C</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>06/2026</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Bullhound Capital, Fynveur, Firgun Ventures</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>9</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Series C</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>06/2026</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Temasek, Intrepid Growth Partners, July Fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>10</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Cambridge Aerospace</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Late VC</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>06/2026</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>DFJ Growth</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>